<commit_message>
Adicionando o grafico com chart
</commit_message>
<xml_diff>
--- a/dados.xlsx
+++ b/dados.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t xml:space="preserve">Ano</t>
+  </si>
   <si>
     <t xml:space="preserve">Titular</t>
   </si>
@@ -110,8 +113,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -307,95 +314,112 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="10.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16380" min="16380" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>129</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>149</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>181</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>28</v>
       </c>
     </row>

</xml_diff>